<commit_message>
feat: update ultrasonic controller and board design
</commit_message>
<xml_diff>
--- a/kicad/ELSONIC/POWER_BD_SV6/POWER_BD_SV6_PL_ALL.xlsx
+++ b/kicad/ELSONIC/POWER_BD_SV6/POWER_BD_SV6_PL_ALL.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01_AllData\06_Embedded_Proj\KiCAD\ELSONIC\POWER_BD_SV6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA8554C2-6D0A-47FD-A007-E3FCC4AEB543}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFE8083-AE69-4B19-B5F4-2F2712386E5F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30525" yWindow="420" windowWidth="24960" windowHeight="15015"/>
+    <workbookView xWindow="3015" yWindow="285" windowWidth="24960" windowHeight="15015" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="POWER_BD_SV5" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="212">
   <si>
     <t>Value</t>
   </si>
@@ -661,7 +661,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1004,7 +1004,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1119,6 +1119,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -1248,8 +1263,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1606,14 +1624,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D66"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F66"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.25" customWidth="1"/>
     <col min="2" max="2" width="18.125" customWidth="1"/>
     <col min="3" max="3" width="57.125" customWidth="1"/>
     <col min="4" max="4" width="17.125" customWidth="1"/>
+    <col min="5" max="5" width="16.75" customWidth="1"/>
+    <col min="6" max="6" width="23.25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -2064,7 +2084,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>111</v>
       </c>
@@ -2078,7 +2098,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>114</v>
       </c>
@@ -2092,7 +2112,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>117</v>
       </c>
@@ -2106,7 +2126,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>120</v>
       </c>
@@ -2120,7 +2140,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>123</v>
       </c>
@@ -2134,7 +2154,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>126</v>
       </c>
@@ -2148,7 +2168,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>129</v>
       </c>
@@ -2162,7 +2182,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>133</v>
       </c>
@@ -2176,7 +2196,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>137</v>
       </c>
@@ -2190,7 +2210,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>140</v>
       </c>
@@ -2204,7 +2224,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>143</v>
       </c>
@@ -2218,7 +2238,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>146</v>
       </c>
@@ -2228,8 +2248,14 @@
       <c r="C44" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E44" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>149</v>
       </c>
@@ -2239,8 +2265,14 @@
       <c r="C45" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E45" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>152</v>
       </c>
@@ -2250,8 +2282,14 @@
       <c r="C46" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E46" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>155</v>
       </c>
@@ -2261,8 +2299,14 @@
       <c r="C47" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E47" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>158</v>
       </c>
@@ -2272,8 +2316,14 @@
       <c r="C48" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E48" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>161</v>
       </c>
@@ -2283,8 +2333,14 @@
       <c r="C49" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E49" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>164</v>
       </c>
@@ -2294,8 +2350,14 @@
       <c r="C50" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E50" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>166</v>
       </c>
@@ -2305,8 +2367,14 @@
       <c r="C51" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E51" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>169</v>
       </c>
@@ -2316,8 +2384,14 @@
       <c r="C52" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E52" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>172</v>
       </c>
@@ -2327,8 +2401,14 @@
       <c r="C53" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E53" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>175</v>
       </c>
@@ -2338,8 +2418,14 @@
       <c r="C54" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E54" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>178</v>
       </c>
@@ -2349,8 +2435,14 @@
       <c r="C55" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E55" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>181</v>
       </c>
@@ -2360,8 +2452,14 @@
       <c r="C56" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E56" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>184</v>
       </c>
@@ -2371,8 +2469,14 @@
       <c r="C57" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E57" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>187</v>
       </c>
@@ -2382,8 +2486,14 @@
       <c r="C58" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E58" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>190</v>
       </c>
@@ -2393,8 +2503,14 @@
       <c r="C59" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E59" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>193</v>
       </c>
@@ -2404,8 +2520,14 @@
       <c r="C60" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E60" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>195</v>
       </c>
@@ -2415,8 +2537,14 @@
       <c r="C61" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E61" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>197</v>
       </c>
@@ -2426,8 +2554,14 @@
       <c r="C62" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E62" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>200</v>
       </c>
@@ -2437,8 +2571,14 @@
       <c r="C63" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E63" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>203</v>
       </c>
@@ -2448,8 +2588,14 @@
       <c r="C64" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E64" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>206</v>
       </c>
@@ -2459,8 +2605,14 @@
       <c r="C65" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E65" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>209</v>
       </c>
@@ -2474,5 +2626,6 @@
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update STM32 firmware, docs, and board design
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kicad/ELSONIC/POWER_BD_SV6/POWER_BD_SV6_PL_ALL.xlsx
+++ b/kicad/ELSONIC/POWER_BD_SV6/POWER_BD_SV6_PL_ALL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01_AllData\06_Embedded_Proj\KiCAD\ELSONIC\POWER_BD_SV6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFE8083-AE69-4B19-B5F4-2F2712386E5F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE3E66A-029A-47D7-987F-24A27B8C9B15}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3015" yWindow="285" windowWidth="24960" windowHeight="15015" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29805" yWindow="360" windowWidth="24960" windowHeight="15015" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="POWER_BD_SV5" sheetId="1" r:id="rId1"/>
@@ -1263,12 +1263,18 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1625,15 +1631,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.25" customWidth="1"/>
     <col min="2" max="2" width="18.125" customWidth="1"/>
     <col min="3" max="3" width="57.125" customWidth="1"/>
     <col min="4" max="4" width="17.125" customWidth="1"/>
-    <col min="5" max="5" width="16.75" customWidth="1"/>
-    <col min="6" max="6" width="23.25" customWidth="1"/>
+    <col min="5" max="5" width="8.875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.375" customWidth="1"/>
+    <col min="7" max="7" width="8.5" style="2" customWidth="1"/>
+    <col min="8" max="8" width="19.25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -2084,7 +2092,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>111</v>
       </c>
@@ -2098,7 +2106,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>114</v>
       </c>
@@ -2112,7 +2120,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>117</v>
       </c>
@@ -2126,7 +2134,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>120</v>
       </c>
@@ -2140,7 +2148,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>123</v>
       </c>
@@ -2154,7 +2162,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>126</v>
       </c>
@@ -2168,7 +2176,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>129</v>
       </c>
@@ -2182,7 +2190,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>133</v>
       </c>
@@ -2196,7 +2204,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>137</v>
       </c>
@@ -2210,7 +2218,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>140</v>
       </c>
@@ -2224,7 +2232,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>143</v>
       </c>
@@ -2238,7 +2246,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>146</v>
       </c>
@@ -2248,14 +2256,20 @@
       <c r="C44" t="s">
         <v>148</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="E44" s="3">
+        <v>1</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="G44" s="3">
+        <v>1</v>
+      </c>
+      <c r="H44" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>149</v>
       </c>
@@ -2265,14 +2279,20 @@
       <c r="C45" t="s">
         <v>151</v>
       </c>
-      <c r="E45" s="1" t="s">
+      <c r="E45" s="3">
+        <v>2</v>
+      </c>
+      <c r="F45" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="G45" s="3">
+        <v>1</v>
+      </c>
+      <c r="H45" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>152</v>
       </c>
@@ -2282,14 +2302,20 @@
       <c r="C46" t="s">
         <v>154</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E46" s="3">
+        <v>3</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="G46" s="3">
+        <v>1</v>
+      </c>
+      <c r="H46" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>155</v>
       </c>
@@ -2299,14 +2325,20 @@
       <c r="C47" t="s">
         <v>157</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="E47" s="3">
+        <v>4</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="G47" s="3">
+        <v>1</v>
+      </c>
+      <c r="H47" s="1" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>158</v>
       </c>
@@ -2316,14 +2348,20 @@
       <c r="C48" t="s">
         <v>160</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="E48" s="3">
+        <v>5</v>
+      </c>
+      <c r="F48" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="G48" s="3">
+        <v>1</v>
+      </c>
+      <c r="H48" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>161</v>
       </c>
@@ -2333,14 +2371,20 @@
       <c r="C49" t="s">
         <v>163</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" s="3">
+        <v>6</v>
+      </c>
+      <c r="F49" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="G49" s="3">
+        <v>1</v>
+      </c>
+      <c r="H49" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>164</v>
       </c>
@@ -2350,14 +2394,20 @@
       <c r="C50" t="s">
         <v>160</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="E50" s="3">
+        <v>7</v>
+      </c>
+      <c r="F50" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="G50" s="3">
+        <v>1</v>
+      </c>
+      <c r="H50" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>166</v>
       </c>
@@ -2367,14 +2417,20 @@
       <c r="C51" t="s">
         <v>168</v>
       </c>
-      <c r="E51" s="1" t="s">
+      <c r="E51" s="3">
+        <v>8</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="G51" s="3">
+        <v>1</v>
+      </c>
+      <c r="H51" s="1" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>169</v>
       </c>
@@ -2384,14 +2440,20 @@
       <c r="C52" t="s">
         <v>171</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E52" s="3">
+        <v>9</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="F52" s="1" t="s">
+      <c r="G52" s="3">
+        <v>1</v>
+      </c>
+      <c r="H52" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>172</v>
       </c>
@@ -2401,14 +2463,20 @@
       <c r="C53" t="s">
         <v>174</v>
       </c>
-      <c r="E53" s="1" t="s">
+      <c r="E53" s="3">
+        <v>10</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="G53" s="3">
+        <v>1</v>
+      </c>
+      <c r="H53" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>175</v>
       </c>
@@ -2418,14 +2486,20 @@
       <c r="C54" t="s">
         <v>177</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="E54" s="3">
+        <v>11</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="G54" s="3">
+        <v>1</v>
+      </c>
+      <c r="H54" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>178</v>
       </c>
@@ -2435,14 +2509,20 @@
       <c r="C55" t="s">
         <v>180</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E55" s="3">
+        <v>12</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="G55" s="3">
+        <v>1</v>
+      </c>
+      <c r="H55" s="1" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>181</v>
       </c>
@@ -2452,14 +2532,20 @@
       <c r="C56" t="s">
         <v>183</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="E56" s="3">
+        <v>13</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="G56" s="3">
+        <v>1</v>
+      </c>
+      <c r="H56" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>184</v>
       </c>
@@ -2469,14 +2555,20 @@
       <c r="C57" t="s">
         <v>186</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="E57" s="3">
+        <v>14</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="G57" s="3">
+        <v>2</v>
+      </c>
+      <c r="H57" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>187</v>
       </c>
@@ -2486,14 +2578,20 @@
       <c r="C58" t="s">
         <v>189</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="E58" s="3">
+        <v>15</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="G58" s="3">
+        <v>1</v>
+      </c>
+      <c r="H58" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>190</v>
       </c>
@@ -2503,14 +2601,20 @@
       <c r="C59" t="s">
         <v>192</v>
       </c>
-      <c r="E59" s="1" t="s">
+      <c r="E59" s="3">
+        <v>16</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="F59" s="1" t="s">
+      <c r="G59" s="3">
+        <v>2</v>
+      </c>
+      <c r="H59" s="1" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>193</v>
       </c>
@@ -2520,14 +2624,20 @@
       <c r="C60" t="s">
         <v>192</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="E60" s="3">
+        <v>17</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="G60" s="3">
+        <v>1</v>
+      </c>
+      <c r="H60" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>195</v>
       </c>
@@ -2537,14 +2647,20 @@
       <c r="C61" t="s">
         <v>192</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="E61" s="3">
+        <v>18</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="G61" s="3">
+        <v>2</v>
+      </c>
+      <c r="H61" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>197</v>
       </c>
@@ -2554,14 +2670,20 @@
       <c r="C62" t="s">
         <v>199</v>
       </c>
-      <c r="E62" s="1" t="s">
+      <c r="E62" s="3">
+        <v>19</v>
+      </c>
+      <c r="F62" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="G62" s="3">
+        <v>1</v>
+      </c>
+      <c r="H62" s="1" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>200</v>
       </c>
@@ -2571,14 +2693,20 @@
       <c r="C63" t="s">
         <v>202</v>
       </c>
-      <c r="E63" s="1" t="s">
+      <c r="E63" s="3">
+        <v>20</v>
+      </c>
+      <c r="F63" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="G63" s="3">
+        <v>1</v>
+      </c>
+      <c r="H63" s="1" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>203</v>
       </c>
@@ -2588,14 +2716,20 @@
       <c r="C64" t="s">
         <v>205</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="E64" s="3">
+        <v>21</v>
+      </c>
+      <c r="F64" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F64" s="1" t="s">
+      <c r="G64" s="3">
+        <v>1</v>
+      </c>
+      <c r="H64" s="1" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>206</v>
       </c>
@@ -2605,14 +2739,20 @@
       <c r="C65" t="s">
         <v>208</v>
       </c>
-      <c r="E65" s="1" t="s">
+      <c r="E65" s="3">
+        <v>22</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="F65" s="1" t="s">
+      <c r="G65" s="3">
+        <v>2</v>
+      </c>
+      <c r="H65" s="1" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>209</v>
       </c>

</xml_diff>